<commit_message>
excess node testing (not working)
</commit_message>
<xml_diff>
--- a/00_code_base/02_unidirectional/output1.xlsx
+++ b/00_code_base/02_unidirectional/output1.xlsx
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>6238.145</v>
+        <v>4.011715132462092</v>
       </c>
     </row>
     <row r="24">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>26.68741541509184</v>
+        <v>122.2770954150918</v>
       </c>
     </row>
     <row r="48">
@@ -1288,7 +1288,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>765.5670206340636</v>
+        <v>669.9773406340637</v>
       </c>
     </row>
     <row r="49">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>95.58967999999999</v>
       </c>
     </row>
     <row r="71">
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>35.70049800800228</v>
+        <v>565.3161041391963</v>
       </c>
     </row>
     <row r="74">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>660.4286259509694</v>
+        <v>35.22333981977535</v>
       </c>
     </row>
     <row r="75">
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>529.615606131194</v>
       </c>
     </row>
     <row r="76">
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>3588.677514628265</v>
+        <v>943.2217443889922</v>
       </c>
     </row>
     <row r="81">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>17.64930959999998</v>
+        <v>17.64930959999999</v>
       </c>
     </row>
     <row r="83">
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>6763.748890998731</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>6138.543604867537</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>6234.133284867537</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -2526,11 +2526,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>('BG', 'MK')</t>
+          <t>('TR', 'BG')</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>3588.677514628265</v>
+        <v>215.12323635</v>
       </c>
     </row>
     <row r="118">
@@ -2544,11 +2544,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>('TR', 'BG')</t>
+          <t>('RU', 'LV')</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>215.12323635</v>
+        <v>0</v>
       </c>
     </row>
     <row r="119">
@@ -2562,11 +2562,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>('RU', 'LV')</t>
+          <t>('LY', 'IT')</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0</v>
+        <v>64.9705</v>
       </c>
     </row>
     <row r="120">
@@ -2580,11 +2580,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>('LY', 'IT')</t>
+          <t>('TN', 'IT')</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>64.9705</v>
+        <v>407.409</v>
       </c>
     </row>
     <row r="121">
@@ -2598,11 +2598,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>('TN', 'IT')</t>
+          <t>('DZ', 'ES')</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>407.409</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>('DZ', 'ES')</t>
+          <t>('MA', 'ES')</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -2634,11 +2634,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>('MA', 'ES')</t>
+          <t>('NO', 'DE')</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0</v>
+        <v>1092.34576309</v>
       </c>
     </row>
     <row r="124">
@@ -2652,11 +2652,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>('NO', 'DE')</t>
+          <t>('NO', 'NL')</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1092.34576309</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>('NO', 'NL')</t>
+          <t>('NO', 'BE')</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>('NO', 'BE')</t>
+          <t>('NO', 'FR')</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>('NO', 'FR')</t>
+          <t>('NO', 'UK')</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>('NO', 'UK')</t>
+          <t>('UK', 'BE')</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0</v>
+        <v>58.55836482884433</v>
       </c>
     </row>
     <row r="129">
@@ -2742,11 +2742,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>('UK', 'BE')</t>
+          <t>('UK', 'NL')</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>58.55836482884433</v>
+        <v>1.307978289999994</v>
       </c>
     </row>
     <row r="130">
@@ -2760,11 +2760,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>('UK', 'NL')</t>
+          <t>('AL', 'IT')</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>1.307978289999994</v>
+        <v>0.277932075</v>
       </c>
     </row>
     <row r="131">
@@ -2778,11 +2778,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>('AL', 'IT')</t>
+          <t>('GR', 'AL')</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0.277932075</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>('GR', 'AL')</t>
+          <t>('TK', 'GR')</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -2814,11 +2814,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>('TK', 'GR')</t>
+          <t>('AL_Prod', 'AL')</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>0</v>
+        <v>0.55586415</v>
       </c>
     </row>
     <row r="134">
@@ -2832,11 +2832,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>('AL_Prod', 'AL')</t>
+          <t>('DZ_Prod', 'DZ')</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.55586415</v>
+        <v>796.255</v>
       </c>
     </row>
     <row r="135">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>('DZ_Prod', 'DZ')</t>
+          <t>('AT_Prod', 'AT')</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>796.255</v>
+        <v>7.56174552</v>
       </c>
     </row>
     <row r="136">
@@ -2868,11 +2868,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>('AT_Prod', 'AT')</t>
+          <t>('BE_Prod', 'BE')</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>7.56174552</v>
+        <v>0.05764300000000001</v>
       </c>
     </row>
     <row r="137">
@@ -2886,11 +2886,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>('BE_Prod', 'BE')</t>
+          <t>('BG_Prod', 'BG')</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.05764300000000001</v>
+        <v>0.53100927</v>
       </c>
     </row>
     <row r="138">
@@ -2904,11 +2904,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>('BG_Prod', 'BG')</t>
+          <t>('HR_Prod', 'HR')</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.53100927</v>
+        <v>8.679521449999999</v>
       </c>
     </row>
     <row r="139">
@@ -2922,11 +2922,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>('HR_Prod', 'HR')</t>
+          <t>('CZ_Prod', 'CZ')</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>8.679521449999999</v>
+        <v>1.91565275</v>
       </c>
     </row>
     <row r="140">
@@ -2940,11 +2940,11 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>('CZ_Prod', 'CZ')</t>
+          <t>('FR_Prod', 'FR')</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>1.91565275</v>
+        <v>0.16949973</v>
       </c>
     </row>
     <row r="141">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>('FR_Prod', 'FR')</t>
+          <t>('GR_Prod', 'GR')</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>0.16949973</v>
+        <v>0.06330960000000002</v>
       </c>
     </row>
     <row r="142">
@@ -2976,11 +2976,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>('GR_Prod', 'GR')</t>
+          <t>('HU_Prod', 'HU')</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0.06330960000000002</v>
+        <v>16.46245</v>
       </c>
     </row>
     <row r="143">
@@ -2994,11 +2994,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>('HU_Prod', 'HU')</t>
+          <t>('IE_Prod', 'IE')</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>16.46245</v>
+        <v>19.82969027</v>
       </c>
     </row>
     <row r="144">
@@ -3012,11 +3012,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>('IE_Prod', 'IE')</t>
+          <t>('RS_Prod', 'RS')</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>19.82969027</v>
+        <v>3.99593</v>
       </c>
     </row>
     <row r="145">
@@ -3030,11 +3030,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>('RS_Prod', 'RS')</t>
+          <t>('SK_Prod', 'SK')</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>3.99593</v>
+        <v>0.6516687699999999</v>
       </c>
     </row>
     <row r="146">
@@ -3048,11 +3048,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>('SK_Prod', 'SK')</t>
+          <t>('SI_Prod', 'SI')</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>0.6516687699999999</v>
+        <v>0.05211318</v>
       </c>
     </row>
     <row r="147">
@@ -3066,11 +3066,11 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>('SI_Prod', 'SI')</t>
+          <t>('TR_Prod', 'TR')</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>0.05211318</v>
+        <v>4.2744727</v>
       </c>
     </row>
     <row r="148">
@@ -3084,11 +3084,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>('TR_Prod', 'TR')</t>
+          <t>('ES_Prod', 'ES')</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>4.2744727</v>
+        <v>0.44942</v>
       </c>
     </row>
     <row r="149">
@@ -3102,11 +3102,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>('ES_Prod', 'ES')</t>
+          <t>('DZ', 'MA')</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0.44942</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150">
@@ -3120,11 +3120,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>('DZ', 'MA')</t>
+          <t>('DZ', 'TN')</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0</v>
+        <v>796.255</v>
       </c>
     </row>
     <row r="151">
@@ -3138,11 +3138,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>('DZ', 'TN')</t>
+          <t>('DK', 'SE')</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>796.255</v>
+        <v>10.747</v>
       </c>
     </row>
     <row r="152">
@@ -3156,11 +3156,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>('DK', 'SE')</t>
+          <t>('RU', 'BY')</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>10.747</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153">
@@ -3174,11 +3174,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>('RU', 'BY')</t>
+          <t>('RU_Prod', 'RU2')</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>0</v>
+        <v>6234.133284867537</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
separate cost for commodity slack
</commit_message>
<xml_diff>
--- a/00_code_base/02_unidirectional/output1.xlsx
+++ b/00_code_base/02_unidirectional/output1.xlsx
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>9049.284665611007</v>
+        <v>88.09608999999999</v>
       </c>
     </row>
     <row r="23">
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>286.261</v>
+        <v>190.67132</v>
       </c>
     </row>
     <row r="27">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>58.55836482884433</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>62.46237265768866</v>
+        <v>194.1225627299879</v>
       </c>
     </row>
     <row r="32">
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>117.1167296576887</v>
       </c>
     </row>
     <row r="35">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>151.2741943994645</v>
+        <v>400.0511141294524</v>
       </c>
     </row>
     <row r="38">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>26.68741541509184</v>
+        <v>122.2770954150918</v>
       </c>
     </row>
     <row r="48">
@@ -1288,7 +1288,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>765.5670206340633</v>
+        <v>669.9773406340635</v>
       </c>
     </row>
     <row r="49">
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>716.4634961296906</v>
+        <v>467.6865763997028</v>
       </c>
     </row>
     <row r="50">
@@ -1378,7 +1378,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>248.7769197299879</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>248.7769197299879</v>
       </c>
     </row>
     <row r="60">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>280.0409197299879</v>
+        <v>31.264</v>
       </c>
     </row>
     <row r="61">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>95.58967999999999</v>
       </c>
     </row>
     <row r="71">
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>696.1291239589713</v>
+        <v>565.3161041391961</v>
       </c>
     </row>
     <row r="74">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>35.22333981977535</v>
       </c>
     </row>
     <row r="75">
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>660.428625950969</v>
+        <v>529.6156061311938</v>
       </c>
     </row>
     <row r="76">
@@ -1864,7 +1864,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>9999.999999999996</v>
+        <v>943.221744388992</v>
       </c>
     </row>
     <row r="81">
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>8925.965235791231</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>58.55836482884433</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>1.307978289999994</v>
+        <v>118.4247079476887</v>
       </c>
     </row>
     <row r="130">
@@ -3178,7 +3178,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>10000</v>
+        <v>6234.133284867537</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
align input data by sources
different sources for EU and non-EU capacities
</commit_message>
<xml_diff>
--- a/00_code_base/02_unidirectional/output1.xlsx
+++ b/00_code_base/02_unidirectional/output1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D150"/>
+  <dimension ref="A1:D140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>191.3207536107825</v>
+        <v>191.3207536107826</v>
       </c>
     </row>
     <row r="24">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>47.07348538384423</v>
+        <v>50.97270794768866</v>
       </c>
     </row>
     <row r="28">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>89.43556376768844</v>
+        <v>89.43556376768842</v>
       </c>
     </row>
     <row r="31">
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>507.2935854776885</v>
+        <v>507.2935854776884</v>
       </c>
     </row>
     <row r="35">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>60.7811822303091</v>
+        <v>125.65052</v>
       </c>
     </row>
     <row r="38">
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>161.2879256991556</v>
+        <v>96.41858792946458</v>
       </c>
     </row>
     <row r="43">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>64.86933776969087</v>
       </c>
     </row>
     <row r="48">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>43.17426281999978</v>
       </c>
     </row>
     <row r="60">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>69.93857844915556</v>
+        <v>5.069240679464585</v>
       </c>
     </row>
     <row r="67">
@@ -1666,7 +1666,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>43.25116303406372</v>
+        <v>43.25116303406362</v>
       </c>
     </row>
     <row r="70">
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.1840311999999962</v>
+        <v>0.3680624000000208</v>
       </c>
     </row>
     <row r="95">
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>3.002865824515279</v>
+        <v>6.005731649030658</v>
       </c>
     </row>
     <row r="97">
@@ -2260,7 +2260,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.277932075</v>
+        <v>0.55586415</v>
       </c>
     </row>
     <row r="103">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>64.9705</v>
+        <v>129.941</v>
       </c>
     </row>
     <row r="108">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>187.3090384783204</v>
+        <v>187.3090384783205</v>
       </c>
     </row>
     <row r="111">
@@ -2436,11 +2436,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>('UA', 'PL')</t>
+          <t>('RU', 'LV')</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.1840311999999962</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>('UA', 'SK')</t>
+          <t>('DZ', 'ES')</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -2472,11 +2472,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>('UA', 'HU')</t>
+          <t>('NO', 'DE')</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>3.002865824515279</v>
+        <v>455.155</v>
       </c>
     </row>
     <row r="115">
@@ -2490,11 +2490,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>('RS', 'HU')</t>
+          <t>('NO', 'NL')</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0</v>
+        <v>351.714</v>
       </c>
     </row>
     <row r="116">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>('BG', 'RS')</t>
+          <t>('NO', 'BE')</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0</v>
+        <v>167.754</v>
       </c>
     </row>
     <row r="117">
@@ -2526,11 +2526,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>('TR', 'BG')</t>
+          <t>('NO', 'FR')</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0</v>
+        <v>117.7227630899998</v>
       </c>
     </row>
     <row r="118">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>('RU', 'LV')</t>
+          <t>('NO', 'UK')</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -2562,11 +2562,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>('LY', 'IT')</t>
+          <t>('UK', 'NL')</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>64.9705</v>
+        <v>67.452</v>
       </c>
     </row>
     <row r="120">
@@ -2580,7 +2580,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>('DZ', 'ES')</t>
+          <t>('GR', 'AL')</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>('MA', 'ES')</t>
+          <t>('DZ', 'MA')</t>
         </is>
       </c>
       <c r="D121" t="n">
@@ -2616,11 +2616,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>('NO', 'DE')</t>
+          <t>('DZ', 'TN')</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>455.155</v>
+        <v>402.647</v>
       </c>
     </row>
     <row r="123">
@@ -2634,11 +2634,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>('NO', 'NL')</t>
+          <t>('DK', 'SE')</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>351.714</v>
+        <v>10.747</v>
       </c>
     </row>
     <row r="124">
@@ -2652,11 +2652,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>('NO', 'BE')</t>
+          <t>('RU', 'BY')</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>167.754</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
@@ -2670,11 +2670,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>('NO', 'FR')</t>
+          <t>('AL_Prod', 'AL')</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>74.54850027000002</v>
+        <v>0.55586415</v>
       </c>
     </row>
     <row r="126">
@@ -2688,11 +2688,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>('NO', 'UK')</t>
+          <t>('DZ_Prod', 'DZ')</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>43.17426281999978</v>
+        <v>402.647</v>
       </c>
     </row>
     <row r="127">
@@ -2706,11 +2706,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>('UK', 'BE')</t>
+          <t>('AT_Prod', 'AT')</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>47.07348538384423</v>
+        <v>7.56174552</v>
       </c>
     </row>
     <row r="128">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>('UK', 'NL')</t>
+          <t>('BE_Prod', 'BE')</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>67.452</v>
+        <v>0.05764300000000001</v>
       </c>
     </row>
     <row r="129">
@@ -2742,11 +2742,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>('AL', 'IT')</t>
+          <t>('BG_Prod', 'BG')</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0.277932075</v>
+        <v>0.53100927</v>
       </c>
     </row>
     <row r="130">
@@ -2760,11 +2760,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>('GR', 'AL')</t>
+          <t>('HR_Prod', 'HR')</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>0</v>
+        <v>8.679521449999999</v>
       </c>
     </row>
     <row r="131">
@@ -2778,11 +2778,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>('AL_Prod', 'AL')</t>
+          <t>('CZ_Prod', 'CZ')</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0.55586415</v>
+        <v>1.91565275</v>
       </c>
     </row>
     <row r="132">
@@ -2796,11 +2796,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>('DZ_Prod', 'DZ')</t>
+          <t>('FR_Prod', 'FR')</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>402.647</v>
+        <v>0.16949973</v>
       </c>
     </row>
     <row r="133">
@@ -2814,11 +2814,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>('AT_Prod', 'AT')</t>
+          <t>('GR_Prod', 'GR')</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>7.56174552</v>
+        <v>0.06330960000000002</v>
       </c>
     </row>
     <row r="134">
@@ -2832,11 +2832,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>('BE_Prod', 'BE')</t>
+          <t>('HU_Prod', 'HU')</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.05764300000000001</v>
+        <v>16.46245</v>
       </c>
     </row>
     <row r="135">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>('BG_Prod', 'BG')</t>
+          <t>('IE_Prod', 'IE')</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>0.53100927</v>
+        <v>19.82969027</v>
       </c>
     </row>
     <row r="136">
@@ -2868,11 +2868,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>('HR_Prod', 'HR')</t>
+          <t>('RS_Prod', 'RS')</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>8.679521449999999</v>
+        <v>3.99593</v>
       </c>
     </row>
     <row r="137">
@@ -2886,11 +2886,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>('CZ_Prod', 'CZ')</t>
+          <t>('SK_Prod', 'SK')</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>1.91565275</v>
+        <v>0.6516687699999999</v>
       </c>
     </row>
     <row r="138">
@@ -2904,11 +2904,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>('FR_Prod', 'FR')</t>
+          <t>('SI_Prod', 'SI')</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.16949973</v>
+        <v>0.05211318</v>
       </c>
     </row>
     <row r="139">
@@ -2922,11 +2922,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>('GR_Prod', 'GR')</t>
+          <t>('TR_Prod', 'TR')</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.06330960000000002</v>
+        <v>4.2744727</v>
       </c>
     </row>
     <row r="140">
@@ -2940,190 +2940,10 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>('HU_Prod', 'HU')</t>
+          <t>('ES_Prod', 'ES')</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>16.46245</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="1" t="n">
-        <v>139</v>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>('IE_Prod', 'IE')</t>
-        </is>
-      </c>
-      <c r="D141" t="n">
-        <v>19.82969027</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="1" t="n">
-        <v>140</v>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>('RS_Prod', 'RS')</t>
-        </is>
-      </c>
-      <c r="D142" t="n">
-        <v>3.99593</v>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="1" t="n">
-        <v>141</v>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>('SK_Prod', 'SK')</t>
-        </is>
-      </c>
-      <c r="D143" t="n">
-        <v>0.6516687699999999</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="1" t="n">
-        <v>142</v>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>('SI_Prod', 'SI')</t>
-        </is>
-      </c>
-      <c r="D144" t="n">
-        <v>0.05211318</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="1" t="n">
-        <v>143</v>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>('TR_Prod', 'TR')</t>
-        </is>
-      </c>
-      <c r="D145" t="n">
-        <v>4.2744727</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="1" t="n">
-        <v>144</v>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>('ES_Prod', 'ES')</t>
-        </is>
-      </c>
-      <c r="D146" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="1" t="n">
-        <v>145</v>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>('DZ', 'MA')</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="1" t="n">
-        <v>146</v>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>('DZ', 'TN')</t>
-        </is>
-      </c>
-      <c r="D148" t="n">
-        <v>402.647</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="1" t="n">
-        <v>147</v>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>('DK', 'SE')</t>
-        </is>
-      </c>
-      <c r="D149" t="n">
-        <v>10.747</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="1" t="n">
-        <v>148</v>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>('RU', 'BY')</t>
-        </is>
-      </c>
-      <c r="D150" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add input data for case variation
</commit_message>
<xml_diff>
--- a/00_code_base/02_unidirectional/output1.xlsx
+++ b/00_code_base/02_unidirectional/output1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D140"/>
+  <dimension ref="A1:D142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>398.454</v>
+        <v>366.0850422333159</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>510.9709999999999</v>
+        <v>464.7096990523113</v>
       </c>
     </row>
     <row r="14">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>47.61897999999999</v>
+        <v>350.61898</v>
       </c>
     </row>
     <row r="17">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>191.3207536107826</v>
+        <v>31.34095756975417</v>
       </c>
     </row>
     <row r="24">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>50.97270794768866</v>
+        <v>4.711407000000022</v>
       </c>
     </row>
     <row r="28">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>89.43556376768842</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>507.2935854776884</v>
+        <v>361.3008267633157</v>
       </c>
     </row>
     <row r="35">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>25.96682367567193</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>85.22750000000001</v>
+        <v>4.288886075671982</v>
       </c>
     </row>
     <row r="42">
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>96.41858792946458</v>
+        <v>306.7052626650919</v>
       </c>
     </row>
     <row r="43">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.04392775030909411</v>
+        <v>4.018324425401111</v>
       </c>
     </row>
     <row r="47">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>64.86933776969087</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>70.6275</v>
+        <v>9.732558905401131</v>
       </c>
     </row>
     <row r="50">
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>3.495004150000028</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>53.62600415000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>3.974396675092017</v>
       </c>
     </row>
     <row r="57">
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>13.75365332490798</v>
+        <v>17.72805</v>
       </c>
     </row>
     <row r="59">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>43.17426281999978</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>81.395</v>
+        <v>31.264</v>
       </c>
     </row>
     <row r="61">
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>5.069240679464585</v>
+        <v>225.5759154150919</v>
       </c>
     </row>
     <row r="67">
@@ -1666,7 +1666,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>43.25116303406362</v>
+        <v>47.0485</v>
       </c>
     </row>
     <row r="70">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>151.84</v>
       </c>
     </row>
     <row r="71">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>1.766001991997733</v>
       </c>
     </row>
     <row r="75">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>81.90600000000001</v>
+        <v>49.53704223331599</v>
       </c>
     </row>
     <row r="92">
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.3680624000000208</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>6.005731649030658</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>85.34556442928984</v>
+        <v>83.5795624372921</v>
       </c>
     </row>
     <row r="98">
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>421.21</v>
+        <v>356.820054755401</v>
       </c>
     </row>
     <row r="107">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>187.3090384783205</v>
+        <v>27.32924243729208</v>
       </c>
     </row>
     <row r="111">
@@ -2422,7 +2422,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>351.714</v>
+        <v>295.1568050533157</v>
       </c>
     </row>
     <row r="116">
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>117.7227630899998</v>
+        <v>56.78645803668405</v>
       </c>
     </row>
     <row r="118">
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>402.647</v>
+        <v>338.257054755401</v>
       </c>
     </row>
     <row r="123">
@@ -2670,11 +2670,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>('AL_Prod', 'AL')</t>
+          <t>('NO', 'DK')</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>0.55586415</v>
+        <v>117.4935</v>
       </c>
     </row>
     <row r="126">
@@ -2688,11 +2688,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>('DZ_Prod', 'DZ')</t>
+          <t>('DK', 'PL')</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>402.647</v>
+        <v>91.52667632432805</v>
       </c>
     </row>
     <row r="127">
@@ -2706,11 +2706,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>('AT_Prod', 'AT')</t>
+          <t>('AL_Prod', 'AL')</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>7.56174552</v>
+        <v>0.55586415</v>
       </c>
     </row>
     <row r="128">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>('BE_Prod', 'BE')</t>
+          <t>('DZ_Prod', 'DZ')</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.05764300000000001</v>
+        <v>338.257054755401</v>
       </c>
     </row>
     <row r="129">
@@ -2742,11 +2742,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>('BG_Prod', 'BG')</t>
+          <t>('AT_Prod', 'AT')</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0.53100927</v>
+        <v>7.56174552</v>
       </c>
     </row>
     <row r="130">
@@ -2760,11 +2760,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>('HR_Prod', 'HR')</t>
+          <t>('BE_Prod', 'BE')</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>8.679521449999999</v>
+        <v>0.05764300000000001</v>
       </c>
     </row>
     <row r="131">
@@ -2778,11 +2778,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>('CZ_Prod', 'CZ')</t>
+          <t>('BG_Prod', 'BG')</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>1.91565275</v>
+        <v>0.53100927</v>
       </c>
     </row>
     <row r="132">
@@ -2796,11 +2796,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>('FR_Prod', 'FR')</t>
+          <t>('HR_Prod', 'HR')</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0.16949973</v>
+        <v>8.679521449999999</v>
       </c>
     </row>
     <row r="133">
@@ -2814,11 +2814,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>('GR_Prod', 'GR')</t>
+          <t>('CZ_Prod', 'CZ')</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>0.06330960000000002</v>
+        <v>1.91565275</v>
       </c>
     </row>
     <row r="134">
@@ -2832,11 +2832,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>('HU_Prod', 'HU')</t>
+          <t>('FR_Prod', 'FR')</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>16.46245</v>
+        <v>0.16949973</v>
       </c>
     </row>
     <row r="135">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>('IE_Prod', 'IE')</t>
+          <t>('GR_Prod', 'GR')</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>19.82969027</v>
+        <v>0.06330960000000002</v>
       </c>
     </row>
     <row r="136">
@@ -2868,11 +2868,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>('RS_Prod', 'RS')</t>
+          <t>('HU_Prod', 'HU')</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>3.99593</v>
+        <v>16.46245</v>
       </c>
     </row>
     <row r="137">
@@ -2886,11 +2886,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>('SK_Prod', 'SK')</t>
+          <t>('IE_Prod', 'IE')</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.6516687699999999</v>
+        <v>19.82969027</v>
       </c>
     </row>
     <row r="138">
@@ -2904,11 +2904,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>('SI_Prod', 'SI')</t>
+          <t>('RS_Prod', 'RS')</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.05211318</v>
+        <v>3.99593</v>
       </c>
     </row>
     <row r="139">
@@ -2922,11 +2922,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>('TR_Prod', 'TR')</t>
+          <t>('SK_Prod', 'SK')</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>4.2744727</v>
+        <v>0.6516687699999999</v>
       </c>
     </row>
     <row r="140">
@@ -2940,10 +2940,46 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
+          <t>('SI_Prod', 'SI')</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>0.05211318</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="1" t="n">
+        <v>139</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>('TR_Prod', 'TR')</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>4.2744727</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="1" t="n">
+        <v>140</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
           <t>('ES_Prod', 'ES')</t>
         </is>
       </c>
-      <c r="D140" t="n">
+      <c r="D142" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update russian case scenarios
</commit_message>
<xml_diff>
--- a/00_code_base/02_unidirectional/output1.xlsx
+++ b/00_code_base/02_unidirectional/output1.xlsx
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>366.0850422333159</v>
+        <v>398.454</v>
       </c>
     </row>
     <row r="12">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>464.7096990523113</v>
+        <v>510.9709999999999</v>
       </c>
     </row>
     <row r="14">
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>350.61898</v>
+        <v>47.61897999999999</v>
       </c>
     </row>
     <row r="17">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>31.34095756975417</v>
+        <v>191.3207536107826</v>
       </c>
     </row>
     <row r="24">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>4.711407000000022</v>
+        <v>50.97270794768866</v>
       </c>
     </row>
     <row r="28">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>25.56806791768847</v>
       </c>
     </row>
     <row r="31">
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>361.3008267633157</v>
+        <v>443.4260896276885</v>
       </c>
     </row>
     <row r="35">
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>306.7052626650919</v>
+        <v>85.83052552946457</v>
       </c>
     </row>
     <row r="43">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.018324425401111</v>
+        <v>0.04392775030909411</v>
       </c>
     </row>
     <row r="47">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>64.86933776969087</v>
       </c>
     </row>
     <row r="48">
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>9.732558905401131</v>
+        <v>70.6275</v>
       </c>
     </row>
     <row r="50">
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>3.495004150000028</v>
       </c>
     </row>
     <row r="51">
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>3.974396675092017</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>17.72805</v>
+        <v>13.75365332490798</v>
       </c>
     </row>
     <row r="59">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>31.264</v>
+        <v>27.76899584999997</v>
       </c>
     </row>
     <row r="61">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>225.5759154150919</v>
+        <v>4.701178279464571</v>
       </c>
     </row>
     <row r="67">
@@ -1666,7 +1666,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>47.0485</v>
+        <v>42.8831006340636</v>
       </c>
     </row>
     <row r="70">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>151.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -1756,7 +1756,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>1.766001991997733</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>49.53704223331599</v>
+        <v>81.90600000000001</v>
       </c>
     </row>
     <row r="92">
@@ -2152,7 +2152,7 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0</v>
+        <v>6.373794049030671</v>
       </c>
     </row>
     <row r="97">
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>83.5795624372921</v>
+        <v>85.34556442928984</v>
       </c>
     </row>
     <row r="98">
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>356.820054755401</v>
+        <v>421.21</v>
       </c>
     </row>
     <row r="107">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>27.32924243729208</v>
+        <v>187.3090384783205</v>
       </c>
     </row>
     <row r="111">
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>295.1568050533157</v>
+        <v>351.714</v>
       </c>
     </row>
     <row r="116">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>167.754</v>
+        <v>147.0607669699998</v>
       </c>
     </row>
     <row r="117">
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>56.78645803668405</v>
+        <v>20.92249612000001</v>
       </c>
     </row>
     <row r="118">
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>338.257054755401</v>
+        <v>402.647</v>
       </c>
     </row>
     <row r="123">
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>338.257054755401</v>
+        <v>402.647</v>
       </c>
     </row>
     <row r="129">

</xml_diff>

<commit_message>
implement storage for peak hour analysis
</commit_message>
<xml_diff>
--- a/00_code_base/02_unidirectional/output1.xlsx
+++ b/00_code_base/02_unidirectional/output1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D149"/>
+  <dimension ref="A1:D143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>425.4823361933159</v>
+        <v>510.9709999999999</v>
       </c>
     </row>
     <row r="14">
@@ -672,11 +672,11 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>('EE_LNG', 'EE')</t>
+          <t>('MA_Prod', 'MA')</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6.657073761334408</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="15">
@@ -690,11 +690,11 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>('FI_LNG', 'FI')</t>
+          <t>('DK_Prod', 'DK')</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>19.54</v>
+        <v>13.94707557</v>
       </c>
     </row>
     <row r="16">
@@ -708,11 +708,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>('DE_LNG', 'DE')</t>
+          <t>('DE_Prod', 'DE')</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>304.824</v>
+        <v>47.61897999999999</v>
       </c>
     </row>
     <row r="17">
@@ -726,11 +726,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>('IE_LNG', 'IE')</t>
+          <t>('IT_Prod', 'IT')</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>24.86409536231131</v>
+        <v>38.41564</v>
       </c>
     </row>
     <row r="18">
@@ -744,11 +744,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>('LV_LNG', 'LV')</t>
+          <t>('LY_Prod', 'LY')</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>11.8009575697542</v>
+        <v>129.941</v>
       </c>
     </row>
     <row r="19">
@@ -762,11 +762,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>('MA_Prod', 'MA')</t>
+          <t>('NL_Prod', 'NL')</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>234.14902171</v>
       </c>
     </row>
     <row r="20">
@@ -780,11 +780,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>('DK_Prod', 'DK')</t>
+          <t>('NO_Prod', 'NO')</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>13.94707557</v>
+        <v>1135.33376309</v>
       </c>
     </row>
     <row r="21">
@@ -798,11 +798,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>('DE_Prod', 'DE')</t>
+          <t>('PL_Prod', 'PL')</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>47.61897999999999</v>
+        <v>54.6424376</v>
       </c>
     </row>
     <row r="22">
@@ -816,11 +816,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>('IT_Prod', 'IT')</t>
+          <t>('RO_Prod', 'RO')</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>38.41564</v>
+        <v>88.09608999999999</v>
       </c>
     </row>
     <row r="23">
@@ -834,11 +834,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>('LY_Prod', 'LY')</t>
+          <t>('RU_Prod', 'RU')</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>129.941</v>
+        <v>97.97782737211696</v>
       </c>
     </row>
     <row r="24">
@@ -852,11 +852,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>('NL_Prod', 'NL')</t>
+          <t>('TN_Prod', 'TN')</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>234.14902171</v>
+        <v>18.563</v>
       </c>
     </row>
     <row r="25">
@@ -870,11 +870,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>('NO_Prod', 'NO')</t>
+          <t>('UK_Prod', 'UK')</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>1135.33376309</v>
+        <v>320.81311304</v>
       </c>
     </row>
     <row r="26">
@@ -888,11 +888,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>('PL_Prod', 'PL')</t>
+          <t>('UA_Prod', 'UA')</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>54.6424376</v>
+        <v>190.67132</v>
       </c>
     </row>
     <row r="27">
@@ -906,11 +906,11 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>('RO_Prod', 'RO')</t>
+          <t>('UK', 'BE')</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>88.09608999999999</v>
+        <v>50.97270794768866</v>
       </c>
     </row>
     <row r="28">
@@ -924,11 +924,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>('RU_Prod', 'RU')</t>
+          <t>('UK', 'IE')</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>5.034405092311314</v>
       </c>
     </row>
     <row r="29">
@@ -942,11 +942,11 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>('TN_Prod', 'TN')</t>
+          <t>('BE', 'UK')</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>18.563</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -960,11 +960,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>('UK_Prod', 'UK')</t>
+          <t>('BE', 'NL')</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>320.81311304</v>
+        <v>89.43556376768842</v>
       </c>
     </row>
     <row r="31">
@@ -978,11 +978,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>('UA_Prod', 'UA')</t>
+          <t>('BE', 'DE')</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>190.67132</v>
+        <v>117.81105</v>
       </c>
     </row>
     <row r="32">
@@ -996,7 +996,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>('UK', 'BE')</t>
+          <t>('BE', 'FR')</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>('UK', 'IE')</t>
+          <t>('NL', 'BE')</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1032,11 +1032,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>('BE', 'UK')</t>
+          <t>('NL', 'DE')</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>507.2935854776884</v>
       </c>
     </row>
     <row r="35">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>('BE', 'NL')</t>
+          <t>('DE', 'BE')</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1068,11 +1068,11 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>('BE', 'DE')</t>
+          <t>('DE', 'NL')</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>88.91140581999977</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1086,11 +1086,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>('BE', 'FR')</t>
+          <t>('DE', 'AT')</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>125.65052</v>
       </c>
     </row>
     <row r="38">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>('NL', 'BE')</t>
+          <t>('DE', 'CH')</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1122,11 +1122,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>('NL', 'DE')</t>
+          <t>('DE', 'FR')</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>388.376470943316</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -1140,11 +1140,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>('DE', 'BE')</t>
+          <t>('DE', 'DK')</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>25.96682367567193</v>
       </c>
     </row>
     <row r="41">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>('DE', 'NL')</t>
+          <t>('DE', 'PL')</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>85.22750000000001</v>
       </c>
     </row>
     <row r="42">
@@ -1176,11 +1176,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>('DE', 'AT')</t>
+          <t>('DE', 'CZ')</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>125.65052</v>
+        <v>196.4185879294646</v>
       </c>
     </row>
     <row r="43">
@@ -1194,11 +1194,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>('DE', 'CH')</t>
+          <t>('DE', 'LU')</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>3.136188022551898</v>
       </c>
     </row>
     <row r="44">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>('DE', 'FR')</t>
+          <t>('AT', 'DE')</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>('DE', 'DK')</t>
+          <t>('AT', 'IT')</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1248,11 +1248,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>('DE', 'PL')</t>
+          <t>('AT', 'SI')</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4.288886075671982</v>
+        <v>2.252322433403378</v>
       </c>
     </row>
     <row r="47">
@@ -1266,11 +1266,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>('DE', 'CZ')</t>
+          <t>('AT', 'SK')</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>306.7052626650919</v>
+        <v>62.66094308659659</v>
       </c>
     </row>
     <row r="48">
@@ -1284,11 +1284,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>('DE', 'LU')</t>
+          <t>('AT', 'HU')</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>3.136188022551898</v>
+        <v>55.8815</v>
       </c>
     </row>
     <row r="49">
@@ -1302,11 +1302,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>('AT', 'DE')</t>
+          <t>('IT', 'AT')</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>70.6275</v>
       </c>
     </row>
     <row r="50">
@@ -1320,11 +1320,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>('AT', 'IT')</t>
+          <t>('IT', 'CH')</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>3.495004150000028</v>
       </c>
     </row>
     <row r="51">
@@ -1338,11 +1338,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>('AT', 'SI')</t>
+          <t>('IT', 'SI')</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4.018324425401111</v>
+        <v>10.4025</v>
       </c>
     </row>
     <row r="52">
@@ -1356,11 +1356,11 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>('AT', 'SK')</t>
+          <t>('CH', 'DE')</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0</v>
+        <v>53.62600415000003</v>
       </c>
     </row>
     <row r="53">
@@ -1374,11 +1374,11 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>('AT', 'HU')</t>
+          <t>('CH', 'IT')</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>55.8815</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -1392,11 +1392,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>('IT', 'AT')</t>
+          <t>('CH', 'FR')</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>9.732558905401131</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>('IT', 'CH')</t>
+          <t>('SI', 'IT')</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1428,11 +1428,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>('IT', 'SI')</t>
+          <t>('SI', 'HR')</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>10.4025</v>
+        <v>2.208394683094284</v>
       </c>
     </row>
     <row r="57">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>('CH', 'DE')</t>
+          <t>('HR', 'SI')</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -1464,11 +1464,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>('CH', 'IT')</t>
+          <t>('HR', 'HU')</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>15.96204800800227</v>
       </c>
     </row>
     <row r="59">
@@ -1482,11 +1482,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>('CH', 'FR')</t>
+          <t>('FR', 'BE')</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>43.17426281999978</v>
       </c>
     </row>
     <row r="60">
@@ -1500,11 +1500,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>('SI', 'IT')</t>
+          <t>('FR', 'CH')</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>81.395</v>
       </c>
     </row>
     <row r="61">
@@ -1518,11 +1518,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>('SI', 'HR')</t>
+          <t>('FR', 'ES')</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>3.974396675092017</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>('HR', 'SI')</t>
+          <t>('DK', 'DE')</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1554,11 +1554,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>('HR', 'HU')</t>
+          <t>('PL', 'DE')</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>17.72805</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
@@ -1572,7 +1572,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>('FR', 'BE')</t>
+          <t>('CZ', 'DE')</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1590,11 +1590,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>('FR', 'CH')</t>
+          <t>('CZ', 'PL')</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>31.264</v>
+        <v>10.22</v>
       </c>
     </row>
     <row r="66">
@@ -1608,11 +1608,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>('FR', 'ES')</t>
+          <t>('CZ', 'SK')</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>105.0692406794646</v>
       </c>
     </row>
     <row r="67">
@@ -1626,7 +1626,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>('DK', 'DE')</t>
+          <t>('SK', 'AT')</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>('PL', 'DE')</t>
+          <t>('SK', 'CZ')</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -1662,11 +1662,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>('CZ', 'DE')</t>
+          <t>('SK', 'HU')</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0</v>
+        <v>47.0485</v>
       </c>
     </row>
     <row r="70">
@@ -1680,11 +1680,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>('CZ', 'PL')</t>
+          <t>('SK', 'UA')</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>93.99426835096935</v>
       </c>
     </row>
     <row r="71">
@@ -1698,11 +1698,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>('CZ', 'SK')</t>
+          <t>('HU', 'HR')</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>225.5759154150919</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>('SK', 'AT')</t>
+          <t>('HU', 'SK')</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -1734,11 +1734,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>('SK', 'CZ')</t>
+          <t>('HU', 'RS')</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0</v>
+        <v>35.70049800800228</v>
       </c>
     </row>
     <row r="74">
@@ -1752,11 +1752,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>('SK', 'HU')</t>
+          <t>('HU', 'RO')</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>47.0485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
@@ -1770,11 +1770,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>('SK', 'UA')</t>
+          <t>('RS', 'BG')</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>151.84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -1788,11 +1788,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>('HU', 'HR')</t>
+          <t>('RS', 'BA')</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="77">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>('HU', 'SK')</t>
+          <t>('BG', 'RS')</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -1824,11 +1824,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>('HU', 'RS')</t>
+          <t>('BG', 'GR')</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>37.46650000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -1842,7 +1842,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>('HU', 'RO')</t>
+          <t>('BG', 'RO')</t>
         </is>
       </c>
       <c r="D79" t="n">
@@ -1860,11 +1860,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>('RS', 'BG')</t>
+          <t>('BG', 'MK')</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>1.766001991997733</v>
+        <v>10.40036286731274</v>
       </c>
     </row>
     <row r="81">
@@ -1878,11 +1878,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>('RS', 'BA')</t>
+          <t>('BG', 'TR')</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>5</v>
+        <v>23.08152729999999</v>
       </c>
     </row>
     <row r="82">
@@ -1896,11 +1896,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>('BG', 'RS')</t>
+          <t>('GR', 'BG')</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0</v>
+        <v>17.64930959999999</v>
       </c>
     </row>
     <row r="83">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>('BG', 'GR')</t>
+          <t>('RO', 'HU')</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -1932,11 +1932,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>('BG', 'RO')</t>
+          <t>('RO', 'BG')</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>0</v>
+        <v>50.12222460951449</v>
       </c>
     </row>
     <row r="85">
@@ -1950,11 +1950,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>('BG', 'MK')</t>
+          <t>('RO', 'UA')</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>10.40036286731274</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -1968,11 +1968,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>('BG', 'TR')</t>
+          <t>('RO', 'MD')</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>23.08152729999999</v>
+        <v>12.91842981977535</v>
       </c>
     </row>
     <row r="87">
@@ -1986,11 +1986,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>('GR', 'BG')</t>
+          <t>('LT', 'LV')</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>17.64930959999999</v>
+        <v>16.21290492348463</v>
       </c>
     </row>
     <row r="88">
@@ -2004,11 +2004,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>('RO', 'HU')</t>
+          <t>('LT', 'RU')</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0</v>
+        <v>8.8712111062035</v>
       </c>
     </row>
     <row r="89">
@@ -2022,11 +2022,11 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>('RO', 'BG')</t>
+          <t>('LV', 'LT')</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>48.35622261751676</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>('RO', 'UA')</t>
+          <t>('LV', 'RU')</t>
         </is>
       </c>
       <c r="D90" t="n">
@@ -2058,11 +2058,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>('RO', 'MD')</t>
+          <t>('ES', 'FR')</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12.91842981977535</v>
+        <v>81.90600000000001</v>
       </c>
     </row>
     <row r="92">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>('LT', 'LV')</t>
+          <t>('ES', 'PT')</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -2094,11 +2094,11 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>('LT', 'RU')</t>
+          <t>('PT', 'ES')</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>25.08411602968813</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -2112,11 +2112,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>('LV', 'LT')</t>
+          <t>('UA', 'PL')</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0</v>
+        <v>0.3680623999999924</v>
       </c>
     </row>
     <row r="95">
@@ -2130,11 +2130,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>('LV', 'RU')</t>
+          <t>('UA', 'SK')</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>2.245126407603976</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -2148,11 +2148,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>('ES', 'FR')</t>
+          <t>('UA', 'HU')</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>81.90600000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -2166,11 +2166,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>('ES', 'PT')</t>
+          <t>('UA', 'RO')</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0</v>
+        <v>85.34556442928984</v>
       </c>
     </row>
     <row r="98">
@@ -2184,7 +2184,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>('PT', 'ES')</t>
+          <t>('MD', 'RO')</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -2202,7 +2202,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>('UA', 'PL')</t>
+          <t>('RU', 'DE')</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>('UA', 'SK')</t>
+          <t>('RU', 'LV')</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -2238,11 +2238,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>('UA', 'HU')</t>
+          <t>('RU', 'FI')</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0</v>
+        <v>19.54</v>
       </c>
     </row>
     <row r="102">
@@ -2256,11 +2256,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>('UA', 'RO')</t>
+          <t>('AL', 'IT')</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>83.57956243729213</v>
+        <v>0.55586415</v>
       </c>
     </row>
     <row r="103">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>('MD', 'RO')</t>
+          <t>('TR', 'BG')</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>('RU', 'DE')</t>
+          <t>('TR', 'GR')</t>
         </is>
       </c>
       <c r="D104" t="n">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>('RU', 'LV')</t>
+          <t>('MA', 'ES')</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -2328,11 +2328,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>('RU', 'FI')</t>
+          <t>('TN', 'IT')</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0</v>
+        <v>421.21</v>
       </c>
     </row>
     <row r="107">
@@ -2346,11 +2346,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>('AL', 'IT')</t>
+          <t>('LY', 'IT')</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.55586415</v>
+        <v>129.941</v>
       </c>
     </row>
     <row r="108">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>('TR', 'BG')</t>
+          <t>('BY', 'PL')</t>
         </is>
       </c>
       <c r="D108" t="n">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>('TR', 'GR')</t>
+          <t>('BY', 'LT')</t>
         </is>
       </c>
       <c r="D109" t="n">
@@ -2400,11 +2400,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>('MA', 'ES')</t>
+          <t>('RU', 'UA')</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0</v>
+        <v>87.30903847832047</v>
       </c>
     </row>
     <row r="111">
@@ -2418,11 +2418,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>('TN', 'IT')</t>
+          <t>('AZ', 'TR')</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>356.820054755401</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="112">
@@ -2436,11 +2436,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>('LY', 'IT')</t>
+          <t>('RU', 'LV')</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>129.941</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -2454,7 +2454,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>('BY', 'PL')</t>
+          <t>('DZ', 'ES')</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -2472,11 +2472,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>('BY', 'LT')</t>
+          <t>('NO', 'DE')</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0</v>
+        <v>455.155</v>
       </c>
     </row>
     <row r="115">
@@ -2490,11 +2490,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>('RU', 'UA')</t>
+          <t>('NO', 'NL')</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>27.32924243729211</v>
+        <v>351.714</v>
       </c>
     </row>
     <row r="116">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>('AZ', 'TR')</t>
+          <t>('NO', 'BE')</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0</v>
+        <v>167.754</v>
       </c>
     </row>
     <row r="117">
@@ -2526,11 +2526,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>('RU', 'LV')</t>
+          <t>('NO', 'FR')</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0</v>
+        <v>117.7227630899998</v>
       </c>
     </row>
     <row r="118">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>('DZ', 'ES')</t>
+          <t>('NO', 'UK')</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -2562,11 +2562,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>('NO', 'DE')</t>
+          <t>('UK', 'NL')</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>455.155</v>
+        <v>67.452</v>
       </c>
     </row>
     <row r="120">
@@ -2580,11 +2580,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>('NO', 'NL')</t>
+          <t>('GR', 'AL')</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>351.714</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121">
@@ -2598,11 +2598,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>('NO', 'BE')</t>
+          <t>('DZ', 'MA')</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>143.5657628199998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="122">
@@ -2616,11 +2616,11 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>('NO', 'FR')</t>
+          <t>('DZ', 'TN')</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>24.41750027000003</v>
+        <v>402.647</v>
       </c>
     </row>
     <row r="123">
@@ -2634,11 +2634,11 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>('NO', 'UK')</t>
+          <t>('DK', 'SE')</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0</v>
+        <v>10.747</v>
       </c>
     </row>
     <row r="124">
@@ -2652,11 +2652,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>('UK', 'NL')</t>
+          <t>('RU', 'BY')</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>37.97044923331595</v>
+        <v>0</v>
       </c>
     </row>
     <row r="125">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>('GR', 'AL')</t>
+          <t>('EE', 'LV')</t>
         </is>
       </c>
       <c r="D125" t="n">
@@ -2688,11 +2688,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>('DZ', 'MA')</t>
+          <t>('LV', 'EE')</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>0</v>
+        <v>6.657073761334408</v>
       </c>
     </row>
     <row r="127">
@@ -2706,11 +2706,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>('DZ', 'TN')</t>
+          <t>('AL_Prod', 'AL')</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>338.257054755401</v>
+        <v>0.55586415</v>
       </c>
     </row>
     <row r="128">
@@ -2724,11 +2724,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>('DK', 'SE')</t>
+          <t>('DZ_Prod', 'DZ')</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>10.747</v>
+        <v>402.647</v>
       </c>
     </row>
     <row r="129">
@@ -2742,11 +2742,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>('RU', 'BY')</t>
+          <t>('AT_Prod', 'AT')</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
+        <v>7.56174552</v>
       </c>
     </row>
     <row r="130">
@@ -2760,11 +2760,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>('NO', 'DK')</t>
+          <t>('BE_Prod', 'BE')</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>117.4935</v>
+        <v>0.05764300000000001</v>
       </c>
     </row>
     <row r="131">
@@ -2778,11 +2778,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>('DK', 'PL')</t>
+          <t>('BG_Prod', 'BG')</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>91.52667632432805</v>
+        <v>0.53100927</v>
       </c>
     </row>
     <row r="132">
@@ -2796,11 +2796,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>('EE', 'LV')</t>
+          <t>('HR_Prod', 'HR')</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>0</v>
+        <v>8.679521449999999</v>
       </c>
     </row>
     <row r="133">
@@ -2814,11 +2814,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>('LV', 'EE')</t>
+          <t>('CZ_Prod', 'CZ')</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>0</v>
+        <v>1.91565275</v>
       </c>
     </row>
     <row r="134">
@@ -2832,11 +2832,11 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>('AL_Prod', 'AL')</t>
+          <t>('FR_Prod', 'FR')</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.55586415</v>
+        <v>0.16949973</v>
       </c>
     </row>
     <row r="135">
@@ -2850,11 +2850,11 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>('DZ_Prod', 'DZ')</t>
+          <t>('GR_Prod', 'GR')</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>338.257054755401</v>
+        <v>0.06330960000000002</v>
       </c>
     </row>
     <row r="136">
@@ -2868,11 +2868,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>('AT_Prod', 'AT')</t>
+          <t>('HU_Prod', 'HU')</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>7.56174552</v>
+        <v>16.46245</v>
       </c>
     </row>
     <row r="137">
@@ -2886,11 +2886,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>('BE_Prod', 'BE')</t>
+          <t>('IE_Prod', 'IE')</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.05764300000000001</v>
+        <v>19.82969027</v>
       </c>
     </row>
     <row r="138">
@@ -2904,11 +2904,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>('BG_Prod', 'BG')</t>
+          <t>('RS_Prod', 'RS')</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>0.53100927</v>
+        <v>3.99593</v>
       </c>
     </row>
     <row r="139">
@@ -2922,11 +2922,11 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>('HR_Prod', 'HR')</t>
+          <t>('SK_Prod', 'SK')</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>8.679521449999999</v>
+        <v>0.6516687699999999</v>
       </c>
     </row>
     <row r="140">
@@ -2940,11 +2940,11 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>('CZ_Prod', 'CZ')</t>
+          <t>('SI_Prod', 'SI')</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>1.91565275</v>
+        <v>0.05211318</v>
       </c>
     </row>
     <row r="141">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>('FR_Prod', 'FR')</t>
+          <t>('TR_Prod', 'TR')</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>0.16949973</v>
+        <v>4.2744727</v>
       </c>
     </row>
     <row r="142">
@@ -2976,11 +2976,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>('GR_Prod', 'GR')</t>
+          <t>('ES_Prod', 'ES')</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>0.06330960000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -2994,119 +2994,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>('HU_Prod', 'HU')</t>
+          <t>('DE_St', 'DE')</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>16.46245</v>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="1" t="n">
-        <v>142</v>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>('IE_Prod', 'IE')</t>
-        </is>
-      </c>
-      <c r="D144" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="1" t="n">
-        <v>143</v>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>('RS_Prod', 'RS')</t>
-        </is>
-      </c>
-      <c r="D145" t="n">
-        <v>3.99593</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="1" t="n">
-        <v>144</v>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>('SK_Prod', 'SK')</t>
-        </is>
-      </c>
-      <c r="D146" t="n">
-        <v>0.6516687699999999</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="1" t="n">
-        <v>145</v>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>('SI_Prod', 'SI')</t>
-        </is>
-      </c>
-      <c r="D147" t="n">
-        <v>0.05211318</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="1" t="n">
-        <v>146</v>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>('TR_Prod', 'TR')</t>
-        </is>
-      </c>
-      <c r="D148" t="n">
-        <v>4.2744727</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="1" t="n">
-        <v>147</v>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>Methane</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>('ES_Prod', 'ES')</t>
-        </is>
-      </c>
-      <c r="D149" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
run model with all storages
</commit_message>
<xml_diff>
--- a/00_code_base/02_unidirectional/output1.xlsx
+++ b/00_code_base/02_unidirectional/output1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D143"/>
+  <dimension ref="A1:D164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,7 +478,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>322.41</v>
+        <v>121.4005</v>
       </c>
     </row>
     <row r="4">
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>73.27499999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>25.402</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>39.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>122.125</v>
+        <v>46.76116424517537</v>
       </c>
     </row>
     <row r="9">
@@ -586,7 +586,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>60.574</v>
+        <v>51.9792424</v>
       </c>
     </row>
     <row r="10">
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>58.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -622,7 +622,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>398.454</v>
+        <v>287.348</v>
       </c>
     </row>
     <row r="12">
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>425.972</v>
+        <v>216.9640290072921</v>
       </c>
     </row>
     <row r="13">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>510.9709999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>13.94707557</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97.97782737211696</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>50.97270794768866</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>89.43556376768842</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>117.81105</v>
+        <v>45.288</v>
       </c>
     </row>
     <row r="32">
@@ -1036,7 +1036,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>507.2935854776884</v>
+        <v>160.4701569928639</v>
       </c>
     </row>
     <row r="35">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>125.65052</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>25.96682367567193</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>85.22750000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>196.4185879294646</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>108.1140285845991</v>
       </c>
     </row>
     <row r="46">
@@ -1252,7 +1252,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2.252322433403378</v>
+        <v>7.635927750309094</v>
       </c>
     </row>
     <row r="47">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>62.66094308659659</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -1288,7 +1288,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>55.8815</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
@@ -1306,7 +1306,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>70.6275</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -1324,7 +1324,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>3.495004150000028</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
@@ -1342,7 +1342,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>10.4025</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>53.62600415000003</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
@@ -1432,7 +1432,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2.208394683094284</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -1450,7 +1450,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>2.8105</v>
       </c>
     </row>
     <row r="58">
@@ -1468,7 +1468,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>15.96204800800227</v>
+        <v>17.72805</v>
       </c>
     </row>
     <row r="59">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>43.17426281999978</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>81.395</v>
+        <v>31.264</v>
       </c>
     </row>
     <row r="61">
@@ -1540,7 +1540,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>1.503435</v>
       </c>
     </row>
     <row r="63">
@@ -1576,7 +1576,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>16.955</v>
       </c>
     </row>
     <row r="65">
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>10.22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>105.0692406794646</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
@@ -1630,7 +1630,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>91.23321081490816</v>
       </c>
     </row>
     <row r="68">
@@ -1666,7 +1666,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>47.0485</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -1684,7 +1684,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>93.99426835096935</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0</v>
+        <v>18.572295</v>
       </c>
     </row>
     <row r="73">
@@ -1738,7 +1738,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>35.70049800800228</v>
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -1774,7 +1774,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>60.30357199199771</v>
       </c>
     </row>
     <row r="76">
@@ -1828,7 +1828,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0</v>
+        <v>42.997</v>
       </c>
     </row>
     <row r="79">
@@ -1882,7 +1882,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>23.08152729999999</v>
+        <v>136.3639709927079</v>
       </c>
     </row>
     <row r="82">
@@ -1900,7 +1900,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>17.64930959999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -1918,7 +1918,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0</v>
+        <v>0.498244999999983</v>
       </c>
     </row>
     <row r="84">
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>50.12222460951449</v>
+        <v>64.27841518022467</v>
       </c>
     </row>
     <row r="85">
@@ -1990,7 +1990,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>16.21290492348463</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
@@ -2008,7 +2008,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>8.8712111062035</v>
+        <v>9.765616029688134</v>
       </c>
     </row>
     <row r="89">
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0</v>
+        <v>23.7615</v>
       </c>
     </row>
     <row r="90">
@@ -2044,7 +2044,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0</v>
+        <v>31.025</v>
       </c>
     </row>
     <row r="91">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>81.90600000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92">
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
+        <v>29.2</v>
       </c>
     </row>
     <row r="94">
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.3680623999999924</v>
+        <v>4.410320000000013</v>
       </c>
     </row>
     <row r="95">
@@ -2170,7 +2170,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>85.34556442928984</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
@@ -2206,7 +2206,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0</v>
+        <v>21.25061602968813</v>
       </c>
     </row>
     <row r="100">
@@ -2260,7 +2260,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.55586415</v>
+        <v>87.86386415</v>
       </c>
     </row>
     <row r="103">
@@ -2332,7 +2332,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>421.21</v>
+        <v>41.26296726540093</v>
       </c>
     </row>
     <row r="107">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>87.30903847832047</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111">
@@ -2422,7 +2422,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>351.714</v>
+        <v>137.1419710376885</v>
       </c>
     </row>
     <row r="116">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>167.754</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117">
@@ -2530,7 +2530,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>117.7227630899998</v>
+        <v>207.5025</v>
       </c>
     </row>
     <row r="118">
@@ -2548,7 +2548,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0</v>
+        <v>292.5462920523113</v>
       </c>
     </row>
     <row r="119">
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>67.452</v>
+        <v>0</v>
       </c>
     </row>
     <row r="120">
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>0</v>
+        <v>87.30799999999999</v>
       </c>
     </row>
     <row r="121">
@@ -2620,7 +2620,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>402.647</v>
+        <v>22.69996726540093</v>
       </c>
     </row>
     <row r="123">
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="D123" t="n">
-        <v>10.747</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124">
@@ -2728,7 +2728,7 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>402.647</v>
+        <v>22.69996726540091</v>
       </c>
     </row>
     <row r="129">
@@ -2764,7 +2764,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>0.05764300000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="131">
@@ -2782,7 +2782,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0.53100927</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
@@ -2800,7 +2800,7 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>8.679521449999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
@@ -2818,7 +2818,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1.91565275</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
@@ -2836,7 +2836,7 @@
         </is>
       </c>
       <c r="D134" t="n">
-        <v>0.16949973</v>
+        <v>0</v>
       </c>
     </row>
     <row r="135">
@@ -2854,7 +2854,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>0.06330960000000002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -2872,7 +2872,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>16.46245</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137">
@@ -2908,7 +2908,7 @@
         </is>
       </c>
       <c r="D138" t="n">
-        <v>3.99593</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
@@ -2926,7 +2926,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0.6516687699999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>4.2744727</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -2998,6 +2998,384 @@
         </is>
       </c>
       <c r="D143" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="1" t="n">
+        <v>142</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>('AT_St', 'AT')</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="1" t="n">
+        <v>143</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>('BE_St', 'BE')</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="1" t="n">
+        <v>144</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>('BG_St', 'BG')</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="1" t="n">
+        <v>145</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>('HR_St', 'HR')</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>40.86641812509202</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="1" t="n">
+        <v>146</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>('CZ_St', 'CZ')</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="1" t="n">
+        <v>147</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>('DK_St', 'DK')</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>30.67033424567192</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="1" t="n">
+        <v>148</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>('FR_St', 'FR')</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="1" t="n">
+        <v>149</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>('GR_St', 'GR')</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="n">
+        <v>150</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>('HU_St', 'HU')</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="1" t="n">
+        <v>151</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>('IT_St', 'IT')</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="1" t="n">
+        <v>152</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>('LV_St', 'LV')</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>70.99940492348463</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="1" t="n">
+        <v>153</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>('NL_St', 'NL')</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="1" t="n">
+        <v>154</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>('PL_St', 'PL')</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="1" t="n">
+        <v>155</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>('PT_St', 'PT')</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>87.81999999999999</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="1" t="n">
+        <v>156</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>('RO_St', 'RO')</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="1" t="n">
+        <v>157</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>('SK_St', 'SK')</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="1" t="n">
+        <v>158</v>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>('SE_St', 'SE')</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>10.747</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="1" t="n">
+        <v>159</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>('RS_St', 'RS')</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="1" t="n">
+        <v>160</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>('TR_St', 'TR')</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="1" t="n">
+        <v>161</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>('UA_St', 'UA')</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="1" t="n">
+        <v>162</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Methane</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>('UK_St', 'UK')</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>